<commit_message>
Bug reports for test project 1
</commit_message>
<xml_diff>
--- a/test-projects/project-1-TodoList/TodoList_Test_cases.xlsx
+++ b/test-projects/project-1-TodoList/TodoList_Test_cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\qa-portfolio\test-projects\project-1-TodoList\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F6BF25A-CD1E-40C7-B06B-98F9D8C4E614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{169D82D1-3321-40AB-8917-AED7B1ACF0C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Munka1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="59">
   <si>
     <t>ID</t>
   </si>
@@ -235,35 +235,6 @@
   </si>
   <si>
     <t>Button is greyed out but the it is still active and can create tasks</t>
-  </si>
-  <si>
-    <t>Test the clear form button with 5 tasks present</t>
-  </si>
-  <si>
-    <t>1.Open the Todolist application
-2.Enter a valid task name
-3.Press the "Create task" button
-4.Repeat steps 2-3 5 times
-5.Press the "Clear form" button</t>
-  </si>
-  <si>
-    <t>The input field is not cleared</t>
-  </si>
-  <si>
-    <t>User can filter if max task amount is reached</t>
-  </si>
-  <si>
-    <t>1.Open the Todolist application
-2.Enter a valid task name
-3.Press the "Create task" button
-4.Repeat steps 2-3 5 times
-5.Press any filter button</t>
-  </si>
-  <si>
-    <t>The filter buttons are not working when 5 or more tasks are present</t>
-  </si>
-  <si>
-    <t>Filter buttons are working correctly</t>
   </si>
 </sst>
 </file>
@@ -324,7 +295,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normál" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
     <dxf>
@@ -365,8 +336,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CD4D7AE9-7053-48D4-B1B3-9C65F11ED91C}" name="TestCaseTable" displayName="TestCaseTable" ref="A1:H19" insertRowShift="1" totalsRowShown="0">
-  <autoFilter ref="A1:H19" xr:uid="{CD4D7AE9-7053-48D4-B1B3-9C65F11ED91C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CD4D7AE9-7053-48D4-B1B3-9C65F11ED91C}" name="TestCaseTable" displayName="TestCaseTable" ref="A1:H17" insertRowShift="1" totalsRowShown="0">
+  <autoFilter ref="A1:H17" xr:uid="{CD4D7AE9-7053-48D4-B1B3-9C65F11ED91C}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{2EB8A0D5-FC6E-4DA5-B0E2-07BBD3D19993}" name="ID" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{9FE3304E-0092-45CA-999F-B24DC69894D6}" name="Summary" dataDxfId="6"/>
@@ -644,7 +615,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" style="1" customWidth="1"/>
@@ -1090,55 +1061,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>17</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>18</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E19" xr:uid="{426B2ADC-AD7E-4BB7-8061-20499878ABF2}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E17" xr:uid="{426B2ADC-AD7E-4BB7-8061-20499878ABF2}">
       <formula1>"TODO,In Progress,Pass,Fail,OKBUT,CNT,Not implemented,Aborted"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>